<commit_message>
docs: sync 2026-09-17 notes, PDF, and master Excel with smart customizer & F&B pillars
</commit_message>
<xml_diff>
--- a/docs/catatan-harian/rekap_catatan_harian.xlsx
+++ b/docs/catatan-harian/rekap_catatan_harian.xlsx
@@ -489,8 +489,8 @@
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="88" customWidth="1" min="3" max="3"/>
-    <col width="99" customWidth="1" min="4" max="4"/>
+    <col width="89" customWidth="1" min="3" max="3"/>
+    <col width="108" customWidth="1" min="4" max="4"/>
     <col width="47" customWidth="1" min="5" max="5"/>
     <col width="23" customWidth="1" min="6" max="6"/>
   </cols>
@@ -505,7 +505,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Master Log Rekapitulasi Harian Pengembang (Sistem Kasir F&amp;B &amp; SaaS Multi-Outlet)</t>
+          <t>Master Log Rekapitulasi Harian Pengembang (Sistem Kasir F&amp;B, KDS, SaaS Multi-Outlet, AI Vision)</t>
         </is>
       </c>
     </row>
@@ -583,17 +583,17 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Major Milestone v2.0 Architecture (SaaS White-Label, QR Code, AI Vision OCR Scanner)</t>
+          <t>Major Milestone v2.0 (SaaS White-Label, QR Code, AI Vision OCR, KDS, HPP &amp; Shift POS)</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>BranchManagerModal.tsx, QRCodeGenerator.tsx, /order page, AiMenuScannerModal.tsx (Tesseract.js)</t>
+          <t>BranchManagerModal, QRCodeGenerator, /order, /kitchen KDS, ingredientActions, shiftActions, productUtils</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>100% SUKSES (Commit: 15e3585 - Live Vercel)</t>
+          <t>100% SUKSES (Commit: 49a9a53 - Live Vercel)</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
@@ -824,27 +824,27 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="72" customWidth="1" min="2" max="2"/>
-    <col width="44" customWidth="1" min="3" max="3"/>
-    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="35" customWidth="1" min="1" max="1"/>
+    <col width="80" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
+    <col width="39" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>📌 CATATAN HARIAN — 17 SEPTEMBER 2026 (v2.0)</t>
+          <t>📌 CATATAN HARIAN — 17 SEPTEMBER 2026 (v2.0 Milestone)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Major Milestone v2.0: White-Label SaaS, QR Code System, &amp; Real AI Vision OCR</t>
+          <t>Penyempurnaan Arsitektur SaaS, QR Ordering, AI OCR, KDS, HPP &amp; Smart Customizer</t>
         </is>
       </c>
     </row>
@@ -987,22 +987,22 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>🧹 OCR 2-Column Unmerger</t>
+          <t>🍳 Kitchen Display System (KDS)</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Memisahkan layout menu 2-kolom &amp; membuang noise brand / footer</t>
+          <t>Live Audio Chime Bell (Web Audio API) &amp; antrean masak/siap/selesai meja</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>AiMenuScannerModal.tsx</t>
+          <t>KitchenDisplayModal.tsx, app/kitchen/page.tsx</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Custom RegEx &amp; Dynamic Line Parser</t>
+          <t>Web Audio API &amp; Next.js</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
@@ -1014,22 +1014,22 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>📦 Batch Import Menu</t>
+          <t>☕ Bahan Baku &amp; HPP (COGS)</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Pratinjau 24 daftar menu bersih lengkap harga &amp; stok + 1-klik simpan</t>
+          <t>Master 11 bahan mentah, resep menu BOM, kalkulasi margin profit &amp; auto-cut</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>AiMenuScannerModal.tsx</t>
+          <t>ingredientActions.ts, AdminView.tsx</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Supabase Batch Insert</t>
+          <t>TypeScript &amp; Next.js Server Actions</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
@@ -1041,25 +1041,79 @@
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>🧾 POS Kasir Customizer</t>
+          <t>💼 Kasir Shift &amp; Cash Drawer</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Support Dine In No. Meja vs Takeaway &amp; kustomisasi rasa pada struk</t>
+          <t>Buka shift kasir, pelacakan kas sistem, rekonsiliasi kas laci &amp; slip closing</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>KasirView.tsx, ReceiptModal.tsx</t>
+          <t>shiftActions.ts, ShiftManagerModal.tsx</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Next.js 16 &amp; React 19</t>
+          <t>Next.js &amp; Thermal 58mm CSS</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>🖨️ Cetak Thermal 58mm &amp; 80mm</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Format cetak struk kasir &amp; Tiket Dapur (KOT) presisi tanpa margin browser</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>ReceiptModal.tsx, KitchenTicketModal.tsx</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>@media print &amp; @page size</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>🧠 Smart Product-Type Customizer</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Pemisahan cerdas: retail tanpa es/gula, makanan level pedas, snack hangat</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>productUtils.ts, order/page.tsx, KasirView.tsx</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>RegEx &amp; Semantic Type Detection</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
         <is>
           <t>Verified</t>
         </is>

</xml_diff>

<commit_message>
feat(pos): dispatch cashier orders to KDS queue with real-time chime & toast alert
</commit_message>
<xml_diff>
--- a/docs/catatan-harian/rekap_catatan_harian.xlsx
+++ b/docs/catatan-harian/rekap_catatan_harian.xlsx
@@ -490,8 +490,8 @@
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
     <col width="89" customWidth="1" min="3" max="3"/>
-    <col width="108" customWidth="1" min="4" max="4"/>
-    <col width="47" customWidth="1" min="5" max="5"/>
+    <col width="105" customWidth="1" min="4" max="4"/>
+    <col width="33" customWidth="1" min="5" max="5"/>
     <col width="23" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -588,12 +588,12 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>BranchManagerModal, QRCodeGenerator, /order, /kitchen KDS, ingredientActions, shiftActions, productUtils</t>
+          <t>BranchManagerModal, QRCodeGenerator, /order, /kitchen KDS, ingredientActions, shiftActions, KasirView</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>100% SUKSES (Commit: 49a9a53 - Live Vercel)</t>
+          <t>100% SUKSES (Live Vercel)</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
@@ -829,7 +829,7 @@
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
     <col width="80" customWidth="1" min="2" max="2"/>
-    <col width="50" customWidth="1" min="3" max="3"/>
+    <col width="64" customWidth="1" min="3" max="3"/>
     <col width="39" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
   </cols>
@@ -987,17 +987,17 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>🍳 Kitchen Display System (KDS)</t>
+          <t>🍳 KDS &amp; Audio Chime Terpadu</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Live Audio Chime Bell (Web Audio API) &amp; antrean masak/siap/selesai meja</t>
+          <t>Live Audio Chime Bell, antrean dapur, notifikasi toast &amp; auto-dispatch kasir</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>KitchenDisplayModal.tsx, app/kitchen/page.tsx</t>
+          <t>KitchenDisplayModal.tsx, app/kitchen/page.tsx, KasirView.tsx</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">

</xml_diff>

<commit_message>
feat(responsive): implement 3-tier adaptive responsive UI for mobile, tablet, and desktop with PWA support
</commit_message>
<xml_diff>
--- a/docs/catatan-harian/rekap_catatan_harian.xlsx
+++ b/docs/catatan-harian/rekap_catatan_harian.xlsx
@@ -824,13 +824,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="80" customWidth="1" min="2" max="2"/>
-    <col width="64" customWidth="1" min="3" max="3"/>
-    <col width="39" customWidth="1" min="4" max="4"/>
+    <col width="98" customWidth="1" min="2" max="2"/>
+    <col width="66" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
@@ -1119,6 +1119,33 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>📱 3-Tier Responsive UI &amp; PWA</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Mobile drawer nav, touch POS catalog, floating bottom bar, bottom sheet checkout, PWA manifest</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>DashboardLayout.tsx, KasirView.tsx, order/page.tsx, layout.tsx</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>CSS Media Queries, React State &amp; PWA</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix(ui): restore clean web-first UI with full vertical scrolling across all modules
</commit_message>
<xml_diff>
--- a/docs/catatan-harian/rekap_catatan_harian.xlsx
+++ b/docs/catatan-harian/rekap_catatan_harian.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rekap Utama" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14 Sep 2026" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17 Sep 2026 (v2.0)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="22 Sep 2026" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -484,8 +485,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <dimension ref="A1:F7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -597,6 +598,36 @@
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>.md, .pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>22 Sep 2026</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Restorasi Web UI Responsif Murni &amp; Optimalisasi Scroll Vertikal (Web-First)</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>DashboardLayout, KasirView, globals.css, QRCodeGenerator, penghapusan kiosk locks</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>100% SUKSES (0 Errors)</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
         <is>
           <t>.md, .pdf</t>
         </is>
@@ -614,7 +645,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
     <col width="87" customWidth="1" min="2" max="2"/>
@@ -825,7 +856,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
     <col width="98" customWidth="1" min="2" max="2"/>
@@ -1149,4 +1180,256 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="31" customWidth="1" min="1" max="1"/>
+    <col width="95" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>📌 CATATAN HARIAN — 22 SEPTEMBER 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Restorasi Web UI Responsif Murni &amp; Optimalisasi Scroll Vertikal Seluruh Modul</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Kategori</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Rincian Pekerjaan &amp; Penyesuaian</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Berkas Terkait</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>Teknologi</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>🎯 Web-First Mandate</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Penegasan prioritas web responsif murni sebelum konversi native sesuai arahan dosen</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Arsitektur Umum</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Metodologi METOPEN</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>🧹 Rollback Kiosk Locks</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Pembersihan overflow:hidden kaku dan bottom sheet tiruan mobile dari commit sebelumnya</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>DashboardLayout.tsx, KasirView.tsx</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>React &amp; CSS</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>📜 Scroll Vertikal Alami</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Aktivasi overflow-y: auto pada tag &lt;main&gt; dan styling scrollbar terracotta di seluruh modul</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>DashboardLayout.tsx, globals.css</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>CSS Webkit Scrollbar</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>📱 Media Queries Responsif</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Pemisahan adaptif desktop (&gt;900px), tablet (&lt;=900px), dan mobile (&lt;=768px) yang fleksibel</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>globals.css, KasirView.tsx</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>CSS Media Queries</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>🖨️ Generator QR Stiker Meja</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Stiker meja dan tombol cetak dapat di-scroll penuh tanpa terpotong di layar laptop</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>QRCodeGenerator.tsx, AdminView.tsx</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>React &amp; qrcode.react</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>🛒 POS Kasir &amp; Pesanan Aktif</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Grid katalog auto-scroll dan ringkasan pesanan aktif selalu presisi</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>KasirView.tsx</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>React State &amp; CSS Grid</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>🔍 Kompilasi Next.js 16</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Build produksi 100% SUKSES tanpa type errors (Turbopack, 9 routes terverifikasi)</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>next build</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Next.js 16 Turbopack</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>100% SUKSES</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: implement 5 lecturer revisions (password reset, HPP modal & low stock warning tone, Google AI Studio vision scanner, and Flutter mobile POS companion)
</commit_message>
<xml_diff>
--- a/docs/catatan-harian/rekap_catatan_harian.xlsx
+++ b/docs/catatan-harian/rekap_catatan_harian.xlsx
@@ -11,6 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14 Sep 2026" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17 Sep 2026 (v2.0)" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="22 Sep 2026" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="26 Sep 2026" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -485,12 +486,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="89" customWidth="1" min="3" max="3"/>
+    <col width="98" customWidth="1" min="3" max="3"/>
     <col width="105" customWidth="1" min="4" max="4"/>
     <col width="33" customWidth="1" min="5" max="5"/>
     <col width="23" customWidth="1" min="6" max="6"/>
@@ -628,6 +629,36 @@
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>.md, .pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>26 Sep 2026</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Mastering Project &amp; Penyelesaian 5 Poin Revisi Dosen (Lupa PW, Pop-up HPP, AI Gemini, Flutter)</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>ResetPasswordClient, HppDetailModal, audioUtils, geminiMenuActions, growkas_mobile</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>100% SUKSES (0 Errors)</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
         <is>
           <t>.md, .pdf</t>
         </is>
@@ -1432,4 +1463,229 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="33" customWidth="1" min="1" max="1"/>
+    <col width="88" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>📌 CATATAN HARIAN — 26 SEPTEMBER 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Mastering Project &amp; Penyelesaian 5 Poin Revisi Dosen Penguji</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Kategori Revisi</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Rincian Pekerjaan &amp; Penyesuaian</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Berkas Terkait</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>Teknologi</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>🔑 1. Lupa &amp; Reset Password</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Alur kirim email reset password Supabase Auth + halaman dedicated /reset-password</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>LoginClient.tsx, authActions.ts, /reset-password</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Supabase Auth</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>💡 2. Pop-up Rincian HPP</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Modal analisis gramasi bahan per porsi, visual ratio bar &amp; indikator margin sehat</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>HppDetailModal.tsx, AdminView.tsx, KasirView.tsx</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>React &amp; TypeScript</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>🔔 2. Audio Bel Stok Menipis</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Web Audio API warning chime (D5 587Hz -&gt; A4 440Hz) saat stok melewati batas minimum</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>audioUtils.ts, AdminView.tsx, KasirView.tsx</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Web Audio API</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>🧠 3. AI Scan Google AI Studio</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Integrasi Gemini 2.0 Flash &amp; 1.5 Pro Multimodal Vision untuk foto menu fisik</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>geminiMenuActions.ts, AiMenuScannerModal.tsx</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Google AI Studio API</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>📱 4. Modul Mobile Flutter</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Aplikasi mobile POS kasir Flutter terhubung ke Supabase &amp; cetak struk Bluetooth 58mm</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>growkas_mobile/ (lib/, pubspec.yaml, README.md)</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Flutter / Dart</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>🔍 5. Mastering &amp; Build</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Kompilasi Next.js 16 Turbopack 100% SUKSES tanpa error (0 errors, 10 rute)</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>next build</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Turbopack</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>100% SUKSES</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
chore: add persistent inventory store seed data and update master academic spreadsheets
</commit_message>
<xml_diff>
--- a/docs/catatan-harian/rekap_catatan_harian.xlsx
+++ b/docs/catatan-harian/rekap_catatan_harian.xlsx
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -56,6 +56,12 @@
       <b val="1"/>
       <color rgb="00166534"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00D4651C"/>
+      <sz val="15"/>
     </font>
   </fonts>
   <fills count="4">
@@ -104,7 +110,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -121,6 +127,7 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -491,7 +498,7 @@
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="98" customWidth="1" min="3" max="3"/>
+    <col width="93" customWidth="1" min="3" max="3"/>
     <col width="105" customWidth="1" min="4" max="4"/>
     <col width="33" customWidth="1" min="5" max="5"/>
     <col width="23" customWidth="1" min="6" max="6"/>
@@ -645,12 +652,12 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Mastering Project &amp; Penyelesaian 5 Poin Revisi Dosen (Lupa PW, Pop-up HPP, AI Gemini, Flutter)</t>
+          <t>Mastering Project, Resiliensi AI Scan Menu (Bypass 503), &amp; Pengurangan Stok HPP Real-Time</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>ResetPasswordClient, HppDetailModal, audioUtils, geminiMenuActions, growkas_mobile</t>
+          <t>geminiMenuActions, ingredientActions, AdminView, KasirView, ResetPasswordClient, growkas_mobile</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
@@ -660,7 +667,7 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>.md, .pdf</t>
+          <t>.md, .pdf, .xlsx</t>
         </is>
       </c>
     </row>
@@ -1471,27 +1478,27 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="33" customWidth="1" min="1" max="1"/>
-    <col width="88" customWidth="1" min="2" max="2"/>
-    <col width="52" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="39" customWidth="1" min="1" max="1"/>
+    <col width="119" customWidth="1" min="2" max="2"/>
+    <col width="56" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>📌 CATATAN HARIAN — 26 SEPTEMBER 2026</t>
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>📌 CATATAN HARIAN PENGEMBANG — 26 SEPTEMBER 2026</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Mastering Project &amp; Penyelesaian 5 Poin Revisi Dosen Penguji</t>
+          <t>Mastering Project, Resiliensi AI Scan Menu (503 Bypass), &amp; Engine Pengurangan Stok HPP Real-Time</t>
         </is>
       </c>
     </row>
@@ -1499,7 +1506,7 @@
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>Kategori Revisi</t>
+          <t>Kategori Revisi / Fitur</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
@@ -1531,7 +1538,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Alur kirim email reset password Supabase Auth + halaman dedicated /reset-password</t>
+          <t>Alur kirim email reset password Supabase Auth + halaman dedicated /reset-password dengan validasi</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -1546,24 +1553,24 @@
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>Verified</t>
+          <t>Verified 100%</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>💡 2. Pop-up Rincian HPP</t>
+          <t>💡 2. Pop-up Rincian HPP (COGS)</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Modal analisis gramasi bahan per porsi, visual ratio bar &amp; indikator margin sehat</t>
+          <t>Modal analisis gramasi bahan baku, visual ratio bar, dan status kesehatan margin (Sehat &gt;=60%, Wajar, Tipis)</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>HppDetailModal.tsx, AdminView.tsx, KasirView.tsx</t>
+          <t>HppDetailModal.tsx, AdminView.tsx</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
@@ -1573,7 +1580,7 @@
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>Verified</t>
+          <t>Verified 100%</t>
         </is>
       </c>
     </row>
@@ -1585,12 +1592,12 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Web Audio API warning chime (D5 587Hz -&gt; A4 440Hz) saat stok melewati batas minimum</t>
+          <t>Web Audio API synthesizer warning chime (D5 587Hz -&gt; A4 440Hz) saat stok melewati batas minimum</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>audioUtils.ts, AdminView.tsx, KasirView.tsx</t>
+          <t>audioUtils.ts, AdminView.tsx</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
@@ -1600,19 +1607,19 @@
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>Verified</t>
+          <t>Verified 100%</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>🧠 3. AI Scan Google AI Studio</t>
+          <t>🧠 3. Resiliensi AI Vision Menu Scan</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Integrasi Gemini 2.0 Flash &amp; 1.5 Pro Multimodal Vision untuk foto menu fisik</t>
+          <t>Multi-model fallback (gemini-flash-latest, 3.8-flash, 3.7-flash, 3.5-flash-lite) bypass error 503 high demand &amp; 404</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -1627,59 +1634,86 @@
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>Verified</t>
+          <t>Verified 100%</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>📱 4. Modul Mobile Flutter</t>
+          <t>📦 4. Pengurangan Stok HPP Real-Time</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Aplikasi mobile POS kasir Flutter terhubung ke Supabase &amp; cetak struk Bluetooth 58mm</t>
+          <t>Live BOM deduction engine saat order kasir/QR, log audit real-time, 3s auto-sync polling, &amp; persistensi disk JSON</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>growkas_mobile/ (lib/, pubspec.yaml, README.md)</t>
+          <t>ingredientActions.ts, orderActions.ts, AdminView.tsx</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Flutter / Dart</t>
+          <t>Next.js Server Actions</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>Verified</t>
+          <t>Verified 100%</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>🔍 5. Mastering &amp; Build</t>
+          <t>📱 5. Modul Mobile Flutter</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Kompilasi Next.js 16 Turbopack 100% SUKSES tanpa error (0 errors, 10 rute)</t>
+          <t>Aplikasi mobile POS kasir Flutter terhubung ke Supabase PostgreSQL &amp; cetak struk Bluetooth 58mm</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
+          <t>growkas/mobile/ (lib/, pubspec.yaml, README.md)</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Flutter / Dart</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>Verified 100%</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>🔍 6. Mastering &amp; Build Turbopack</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Kompilasi Next.js 16 Turbopack 100% SUKSES tanpa error (0 errors, 10 rute Next.js aktif)</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
           <t>next build</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="D11" s="5" t="inlineStr">
         <is>
           <t>Turbopack</t>
         </is>
       </c>
-      <c r="E10" s="6" t="inlineStr">
+      <c r="E11" s="6" t="inlineStr">
         <is>
           <t>100% SUKSES</t>
         </is>

</xml_diff>

<commit_message>
feat: implement modifier-aware HPP stock deduction and fix Vercel HPP pop-up crash
</commit_message>
<xml_diff>
--- a/docs/catatan-harian/rekap_catatan_harian.xlsx
+++ b/docs/catatan-harian/rekap_catatan_harian.xlsx
@@ -1478,12 +1478,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="39" customWidth="1" min="1" max="1"/>
-    <col width="119" customWidth="1" min="2" max="2"/>
-    <col width="56" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="152" customWidth="1" min="2" max="2"/>
+    <col width="61" customWidth="1" min="3" max="3"/>
     <col width="26" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
   </cols>
@@ -1695,25 +1695,52 @@
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>🔍 6. Mastering &amp; Build Turbopack</t>
+          <t>🎯 7. Modifier-Aware HPP &amp; Vercel Fix</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
+          <t>Pengurangan stok adaptif kustomisasi (Less Sugar -50%, No Sugar 0%, No Ice +20% susu, Extra Shot +18g), fix Vercel /tmp path &amp; item_cost null-safety</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>ingredientActions.ts, storeManager.ts, HppDetailModal.tsx</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Next.js &amp; TypeScript</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>Verified 100%</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>🔍 8. Mastering &amp; Build Turbopack</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
           <t>Kompilasi Next.js 16 Turbopack 100% SUKSES tanpa error (0 errors, 10 rute Next.js aktif)</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C12" s="5" t="inlineStr">
         <is>
           <t>next build</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="D12" s="5" t="inlineStr">
         <is>
           <t>Turbopack</t>
         </is>
       </c>
-      <c r="E11" s="6" t="inlineStr">
+      <c r="E12" s="6" t="inlineStr">
         <is>
           <t>100% SUKSES</t>
         </is>

</xml_diff>

<commit_message>
feat: database kosongan, modal input manual stok, dan editor takaran resep modifier
</commit_message>
<xml_diff>
--- a/docs/catatan-harian/rekap_catatan_harian.xlsx
+++ b/docs/catatan-harian/rekap_catatan_harian.xlsx
@@ -1478,12 +1478,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
     <col width="152" customWidth="1" min="2" max="2"/>
-    <col width="61" customWidth="1" min="3" max="3"/>
+    <col width="90" customWidth="1" min="3" max="3"/>
     <col width="26" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
   </cols>
@@ -1746,6 +1746,33 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>🧹 9. Form Stok &amp; Editor Modifier</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Database kosongan zero-baseline, modal input/set stok fisik manual, modal konfigurasi resep normal &amp; rasio takaran modifier (Sugar, Ice, Spicy)</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>IngredientFormModal.tsx, RecipeModifierEditorModal.tsx, AdminView.tsx, storeManager.ts</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Next.js &amp; React</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>Verified 100%</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: sinkronisasi global multi-outlet antara header dropdown dan tab filter admin, master store cabang persisten, serta modal kelola cabang
</commit_message>
<xml_diff>
--- a/docs/catatan-harian/rekap_catatan_harian.xlsx
+++ b/docs/catatan-harian/rekap_catatan_harian.xlsx
@@ -1478,12 +1478,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
     <col width="152" customWidth="1" min="2" max="2"/>
-    <col width="90" customWidth="1" min="3" max="3"/>
+    <col width="118" customWidth="1" min="3" max="3"/>
     <col width="26" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
   </cols>
@@ -1773,6 +1773,33 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>🏪 10. Sinkronisasi Multi-Outlet</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Sinkronisasi two-way dropdown header atas &amp; tab filter admin, master store cabang persisten, auto-deduplikasi, dan modal kelola/hapus cabang</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>DashboardClient.tsx, DashboardLayout.tsx, AdminView.tsx, BranchManagerModal.tsx, branchActions.ts, storeManager.ts</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Next.js &amp; TypeScript</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>Verified 100%</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: diferensiasi katalog menu, resep HPP, dan navigasi multi-brand Saray vs 7co
</commit_message>
<xml_diff>
--- a/docs/catatan-harian/rekap_catatan_harian.xlsx
+++ b/docs/catatan-harian/rekap_catatan_harian.xlsx
@@ -1478,11 +1478,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="152" customWidth="1" min="2" max="2"/>
+    <col width="41" customWidth="1" min="1" max="1"/>
+    <col width="162" customWidth="1" min="2" max="2"/>
     <col width="118" customWidth="1" min="3" max="3"/>
     <col width="26" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
@@ -1800,6 +1800,33 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>🏢 11. Diferensiasi Brand Saray vs 7co</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Pemisahan menu POS Kasir, banner brand dinamis, 17 menu specialty 7co, 7 resep BOM HPP baru, badge Saray/7co di tabel HPP, dan ranking produk terlaris adaptif</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>storeManager.ts, KasirView.tsx, AdminView.tsx, ingredientActions.ts, growkas_master_store.json</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Next.js &amp; Turbopack</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>Verified 100%</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: pruning seluruh cabang dan fokus murni ke 1 outlet tunggal 7co Yogyakarta
</commit_message>
<xml_diff>
--- a/docs/catatan-harian/rekap_catatan_harian.xlsx
+++ b/docs/catatan-harian/rekap_catatan_harian.xlsx
@@ -1478,7 +1478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="41" customWidth="1" min="1" max="1"/>
@@ -1827,6 +1827,33 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>🎯 12. Fokus 1 Outlet Tunggal 7co</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Pruning seluruh cabang sampel non-aktif, menetapkan 7co Yogyakarta sebagai outlet tunggal, proteksi deletion cabang tunggal, dan isolasi katalog murni 7co</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>storeManager.ts, growkas_master_store.json, DashboardClient.tsx, DashboardLayout.tsx, AdminView.tsx</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Next.js &amp; TypeScript</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="inlineStr">
+        <is>
+          <t>Verified 100%</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>